<commit_message>
docs: refresh verified April evidence
</commit_message>
<xml_diff>
--- a/outputs/2026-04/healthcare_ops_kpi_qa_pack_2026_04.xlsx
+++ b/outputs/2026-04/healthcare_ops_kpi_qa_pack_2026_04.xlsx
@@ -707,7 +707,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="18" customHeight="1"/>
   <cols>
     <col min="1" max="11" width="18.7109375" customWidth="1"/>
@@ -862,8 +862,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1">
-      <c r="A12" s="1" t="s">
-        <v>110</v>
+      <c r="A12" t="s">
+        <v>13</v>
       </c>
       <c r="B12">
         <v>0.8</v>
@@ -878,43 +878,48 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="18" customHeight="1">
-      <c r="A13" t="s">
-        <v>15</v>
-      </c>
-    </row>
     <row r="14" spans="1:5" ht="18" customHeight="1">
-      <c r="A14" t="s">
-        <v>16</v>
+      <c r="A14" s="1" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="18" customHeight="1">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="18" customHeight="1">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="18" customHeight="1">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="18" customHeight="1">
       <c r="A20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="18" customHeight="1">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="18" customHeight="1">
+      <c r="A22" t="s">
         <v>22</v>
       </c>
     </row>
@@ -983,7 +988,7 @@
     </row>
     <row r="2" spans="1:16" ht="18" customHeight="1">
       <c r="A2">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B2">
         <v>20260430</v>
@@ -1015,7 +1020,7 @@
     </row>
     <row r="3" spans="1:16" ht="18" customHeight="1">
       <c r="A3">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B3">
         <v>20260430</v>
@@ -1047,7 +1052,7 @@
     </row>
     <row r="4" spans="1:16" ht="18" customHeight="1">
       <c r="A4">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B4">
         <v>20260430</v>
@@ -1082,7 +1087,7 @@
     </row>
     <row r="5" spans="1:16" ht="18" customHeight="1">
       <c r="A5">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B5">
         <v>20260430</v>
@@ -1114,7 +1119,7 @@
     </row>
     <row r="6" spans="1:16" ht="18" customHeight="1">
       <c r="A6">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B6">
         <v>20260430</v>
@@ -1146,7 +1151,7 @@
     </row>
     <row r="7" spans="1:16" ht="18" customHeight="1">
       <c r="A7">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B7">
         <v>20260430</v>
@@ -1178,7 +1183,7 @@
     </row>
     <row r="8" spans="1:16" ht="18" customHeight="1">
       <c r="A8">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B8">
         <v>20260430</v>
@@ -1213,7 +1218,7 @@
     </row>
     <row r="9" spans="1:16" ht="18" customHeight="1">
       <c r="A9">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B9">
         <v>20260430</v>
@@ -1248,7 +1253,7 @@
     </row>
     <row r="10" spans="1:16" ht="18" customHeight="1">
       <c r="A10">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B10">
         <v>20260430</v>
@@ -1283,7 +1288,7 @@
     </row>
     <row r="11" spans="1:16" ht="18" customHeight="1">
       <c r="A11">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B11">
         <v>20260430</v>
@@ -1292,7 +1297,7 @@
         <v>1</v>
       </c>
       <c r="D11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -1321,7 +1326,7 @@
     </row>
     <row r="12" spans="1:16" ht="18" customHeight="1">
       <c r="A12">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B12">
         <v>20260430</v>
@@ -1330,7 +1335,7 @@
         <v>2</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -1359,7 +1364,7 @@
     </row>
     <row r="13" spans="1:16" ht="18" customHeight="1">
       <c r="A13">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B13">
         <v>20260430</v>
@@ -1368,7 +1373,7 @@
         <v>3</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -1400,7 +1405,7 @@
     </row>
     <row r="14" spans="1:16" ht="18" customHeight="1">
       <c r="A14">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B14">
         <v>20260430</v>
@@ -1409,7 +1414,7 @@
         <v>4</v>
       </c>
       <c r="D14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -1438,7 +1443,7 @@
     </row>
     <row r="15" spans="1:16" ht="18" customHeight="1">
       <c r="A15">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B15">
         <v>20260430</v>
@@ -1447,7 +1452,7 @@
         <v>5</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -1473,7 +1478,7 @@
     </row>
     <row r="16" spans="1:16" ht="18" customHeight="1">
       <c r="A16">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B16">
         <v>20260430</v>
@@ -1482,7 +1487,7 @@
         <v>6</v>
       </c>
       <c r="D16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -1508,7 +1513,7 @@
     </row>
     <row r="17" spans="1:15" ht="18" customHeight="1">
       <c r="A17">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B17">
         <v>20260430</v>
@@ -1517,7 +1522,7 @@
         <v>7</v>
       </c>
       <c r="D17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -1546,7 +1551,7 @@
     </row>
     <row r="18" spans="1:15" ht="18" customHeight="1">
       <c r="A18">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B18">
         <v>20260430</v>
@@ -1555,7 +1560,7 @@
         <v>8</v>
       </c>
       <c r="D18">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F18">
         <v>1</v>
@@ -1587,7 +1592,7 @@
     </row>
     <row r="19" spans="1:15" ht="18" customHeight="1">
       <c r="A19">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B19">
         <v>20260430</v>
@@ -1596,7 +1601,7 @@
         <v>9</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F19">
         <v>1</v>
@@ -1628,7 +1633,7 @@
     </row>
     <row r="20" spans="1:15" ht="18" customHeight="1">
       <c r="A20">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B20">
         <v>20260430</v>
@@ -1666,7 +1671,7 @@
     </row>
     <row r="21" spans="1:15" ht="18" customHeight="1">
       <c r="A21">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B21">
         <v>20260430</v>
@@ -1701,7 +1706,7 @@
     </row>
     <row r="22" spans="1:15" ht="18" customHeight="1">
       <c r="A22">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B22">
         <v>20260430</v>
@@ -1739,7 +1744,7 @@
     </row>
     <row r="23" spans="1:15" ht="18" customHeight="1">
       <c r="A23">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B23">
         <v>20260430</v>
@@ -1774,7 +1779,7 @@
     </row>
     <row r="24" spans="1:15" ht="18" customHeight="1">
       <c r="A24">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B24">
         <v>20260430</v>
@@ -1812,7 +1817,7 @@
     </row>
     <row r="25" spans="1:15" ht="18" customHeight="1">
       <c r="A25">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B25">
         <v>20260430</v>
@@ -1847,7 +1852,7 @@
     </row>
     <row r="26" spans="1:15" ht="18" customHeight="1">
       <c r="A26">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B26">
         <v>20260430</v>
@@ -1885,7 +1890,7 @@
     </row>
     <row r="27" spans="1:15" ht="18" customHeight="1">
       <c r="A27">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B27">
         <v>20260430</v>
@@ -1926,7 +1931,7 @@
     </row>
     <row r="28" spans="1:15" ht="18" customHeight="1">
       <c r="A28">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B28">
         <v>20260430</v>
@@ -1967,7 +1972,7 @@
     </row>
     <row r="29" spans="1:15" ht="18" customHeight="1">
       <c r="A29">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B29">
         <v>20260430</v>
@@ -2005,7 +2010,7 @@
     </row>
     <row r="30" spans="1:15" ht="18" customHeight="1">
       <c r="A30">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B30">
         <v>20260430</v>
@@ -2040,7 +2045,7 @@
     </row>
     <row r="31" spans="1:15" ht="18" customHeight="1">
       <c r="A31">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B31">
         <v>20260430</v>
@@ -2078,7 +2083,7 @@
     </row>
     <row r="32" spans="1:15" ht="18" customHeight="1">
       <c r="A32">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B32">
         <v>20260430</v>
@@ -2113,7 +2118,7 @@
     </row>
     <row r="33" spans="1:16" ht="18" customHeight="1">
       <c r="A33">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B33">
         <v>20260430</v>
@@ -2151,7 +2156,7 @@
     </row>
     <row r="34" spans="1:16" ht="18" customHeight="1">
       <c r="A34">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B34">
         <v>20260430</v>
@@ -2186,7 +2191,7 @@
     </row>
     <row r="35" spans="1:16" ht="18" customHeight="1">
       <c r="A35">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B35">
         <v>20260430</v>
@@ -2224,7 +2229,7 @@
     </row>
     <row r="36" spans="1:16" ht="18" customHeight="1">
       <c r="A36">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B36">
         <v>20260430</v>
@@ -2262,7 +2267,7 @@
     </row>
     <row r="37" spans="1:16" ht="18" customHeight="1">
       <c r="A37">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B37">
         <v>20260430</v>
@@ -2300,7 +2305,7 @@
     </row>
     <row r="38" spans="1:16" ht="18" customHeight="1">
       <c r="A38">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B38">
         <v>20260430</v>
@@ -2309,7 +2314,7 @@
         <v>1</v>
       </c>
       <c r="D38">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F38">
         <v>2</v>
@@ -2338,7 +2343,7 @@
     </row>
     <row r="39" spans="1:16" ht="18" customHeight="1">
       <c r="A39">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B39">
         <v>20260430</v>
@@ -2347,7 +2352,7 @@
         <v>2</v>
       </c>
       <c r="D39">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F39">
         <v>1</v>
@@ -2376,7 +2381,7 @@
     </row>
     <row r="40" spans="1:16" ht="18" customHeight="1">
       <c r="A40">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B40">
         <v>20260430</v>
@@ -2385,7 +2390,7 @@
         <v>3</v>
       </c>
       <c r="D40">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F40">
         <v>0.5</v>
@@ -2417,7 +2422,7 @@
     </row>
     <row r="41" spans="1:16" ht="18" customHeight="1">
       <c r="A41">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B41">
         <v>20260430</v>
@@ -2426,7 +2431,7 @@
         <v>4</v>
       </c>
       <c r="D41">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F41">
         <v>5</v>
@@ -2455,7 +2460,7 @@
     </row>
     <row r="42" spans="1:16" ht="18" customHeight="1">
       <c r="A42">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B42">
         <v>20260430</v>
@@ -2464,7 +2469,7 @@
         <v>5</v>
       </c>
       <c r="D42">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F42">
         <v>1</v>
@@ -2493,7 +2498,7 @@
     </row>
     <row r="43" spans="1:16" ht="18" customHeight="1">
       <c r="A43">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B43">
         <v>20260430</v>
@@ -2502,7 +2507,7 @@
         <v>6</v>
       </c>
       <c r="D43">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -2531,7 +2536,7 @@
     </row>
     <row r="44" spans="1:16" ht="18" customHeight="1">
       <c r="A44">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B44">
         <v>20260430</v>
@@ -2540,7 +2545,7 @@
         <v>7</v>
       </c>
       <c r="D44">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F44">
         <v>0.5</v>
@@ -2572,7 +2577,7 @@
     </row>
     <row r="45" spans="1:16" ht="18" customHeight="1">
       <c r="A45">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B45">
         <v>20260430</v>
@@ -2581,7 +2586,7 @@
         <v>8</v>
       </c>
       <c r="D45">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F45">
         <v>1</v>
@@ -2613,7 +2618,7 @@
     </row>
     <row r="46" spans="1:16" ht="18" customHeight="1">
       <c r="A46">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B46">
         <v>20260430</v>
@@ -2622,7 +2627,7 @@
         <v>9</v>
       </c>
       <c r="D46">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F46">
         <v>1</v>
@@ -2654,7 +2659,7 @@
     </row>
     <row r="47" spans="1:16" ht="18" customHeight="1">
       <c r="A47">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B47">
         <v>20260430</v>
@@ -2692,7 +2697,7 @@
     </row>
     <row r="48" spans="1:16" ht="18" customHeight="1">
       <c r="A48">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B48">
         <v>20260430</v>
@@ -2730,7 +2735,7 @@
     </row>
     <row r="49" spans="1:16" ht="18" customHeight="1">
       <c r="A49">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B49">
         <v>20260430</v>
@@ -2771,7 +2776,7 @@
     </row>
     <row r="50" spans="1:16" ht="18" customHeight="1">
       <c r="A50">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B50">
         <v>20260430</v>
@@ -2809,7 +2814,7 @@
     </row>
     <row r="51" spans="1:16" ht="18" customHeight="1">
       <c r="A51">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B51">
         <v>20260430</v>
@@ -2847,7 +2852,7 @@
     </row>
     <row r="52" spans="1:16" ht="18" customHeight="1">
       <c r="A52">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B52">
         <v>20260430</v>
@@ -2885,7 +2890,7 @@
     </row>
     <row r="53" spans="1:16" ht="18" customHeight="1">
       <c r="A53">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B53">
         <v>20260430</v>
@@ -2926,7 +2931,7 @@
     </row>
     <row r="54" spans="1:16" ht="18" customHeight="1">
       <c r="A54">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B54">
         <v>20260430</v>
@@ -2967,7 +2972,7 @@
     </row>
     <row r="55" spans="1:16" ht="18" customHeight="1">
       <c r="A55">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B55">
         <v>20260430</v>
@@ -3008,7 +3013,7 @@
     </row>
     <row r="56" spans="1:16" ht="18" customHeight="1">
       <c r="A56">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B56">
         <v>20260430</v>
@@ -3046,7 +3051,7 @@
     </row>
     <row r="57" spans="1:16" ht="18" customHeight="1">
       <c r="A57">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B57">
         <v>20260430</v>
@@ -3081,7 +3086,7 @@
     </row>
     <row r="58" spans="1:16" ht="18" customHeight="1">
       <c r="A58">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B58">
         <v>20260430</v>
@@ -3119,7 +3124,7 @@
     </row>
     <row r="59" spans="1:16" ht="18" customHeight="1">
       <c r="A59">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B59">
         <v>20260430</v>
@@ -3154,7 +3159,7 @@
     </row>
     <row r="60" spans="1:16" ht="18" customHeight="1">
       <c r="A60">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B60">
         <v>20260430</v>
@@ -3192,7 +3197,7 @@
     </row>
     <row r="61" spans="1:16" ht="18" customHeight="1">
       <c r="A61">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B61">
         <v>20260430</v>
@@ -3227,7 +3232,7 @@
     </row>
     <row r="62" spans="1:16" ht="18" customHeight="1">
       <c r="A62">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B62">
         <v>20260430</v>
@@ -3265,7 +3270,7 @@
     </row>
     <row r="63" spans="1:16" ht="18" customHeight="1">
       <c r="A63">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B63">
         <v>20260430</v>
@@ -3306,7 +3311,7 @@
     </row>
     <row r="64" spans="1:16" ht="18" customHeight="1">
       <c r="A64">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B64">
         <v>20260430</v>
@@ -3347,7 +3352,7 @@
     </row>
     <row r="65" spans="1:16" ht="18" customHeight="1">
       <c r="A65">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B65">
         <v>20260430</v>
@@ -3385,7 +3390,7 @@
     </row>
     <row r="66" spans="1:16" ht="18" customHeight="1">
       <c r="A66">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B66">
         <v>20260430</v>
@@ -3423,7 +3428,7 @@
     </row>
     <row r="67" spans="1:16" ht="18" customHeight="1">
       <c r="A67">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B67">
         <v>20260430</v>
@@ -3464,7 +3469,7 @@
     </row>
     <row r="68" spans="1:16" ht="18" customHeight="1">
       <c r="A68">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B68">
         <v>20260430</v>
@@ -3502,7 +3507,7 @@
     </row>
     <row r="69" spans="1:16" ht="18" customHeight="1">
       <c r="A69">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B69">
         <v>20260430</v>
@@ -3537,7 +3542,7 @@
     </row>
     <row r="70" spans="1:16" ht="18" customHeight="1">
       <c r="A70">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B70">
         <v>20260430</v>
@@ -3572,7 +3577,7 @@
     </row>
     <row r="71" spans="1:16" ht="18" customHeight="1">
       <c r="A71">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B71">
         <v>20260430</v>
@@ -3610,7 +3615,7 @@
     </row>
     <row r="72" spans="1:16" ht="18" customHeight="1">
       <c r="A72">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B72">
         <v>20260430</v>
@@ -3651,7 +3656,7 @@
     </row>
     <row r="73" spans="1:16" ht="18" customHeight="1">
       <c r="A73">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B73">
         <v>20260430</v>
@@ -5191,16 +5196,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6" t="s">
         <v>52</v>
@@ -5251,16 +5256,16 @@
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9" t="s">
         <v>52</v>
@@ -5348,10 +5353,10 @@
         <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D14">
-        <v>0.3333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -5408,10 +5413,10 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D17">
-        <v>0.6666666666666666</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -5505,16 +5510,16 @@
         <v>9</v>
       </c>
       <c r="B22" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D22">
-        <v>0.6666666666666666</v>
+        <v>1.333333333333333</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22" t="s">
         <v>52</v>
@@ -5565,16 +5570,16 @@
         <v>9</v>
       </c>
       <c r="B25" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D25">
-        <v>1.333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25" t="s">
         <v>52</v>
@@ -5662,16 +5667,16 @@
         <v>10</v>
       </c>
       <c r="B30" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" t="s">
         <v>52</v>
@@ -5722,16 +5727,16 @@
         <v>10</v>
       </c>
       <c r="B33" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33" t="s">
         <v>52</v>
@@ -5763,7 +5768,7 @@
         <v>23</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18" customHeight="1">
@@ -5902,13 +5907,13 @@
     </row>
     <row r="2" spans="1:9" ht="18" customHeight="1">
       <c r="A2">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B2">
-        <v>7</v>
+        <v>145</v>
       </c>
       <c r="C2">
-        <v>30</v>
+        <v>628</v>
       </c>
       <c r="D2" t="s">
         <v>79</v>
@@ -5926,18 +5931,18 @@
         <v>107</v>
       </c>
       <c r="I2" s="3">
-        <v>46234.23118008608</v>
+        <v>46244.73807913656</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="18" customHeight="1">
       <c r="A3">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>145</v>
       </c>
       <c r="C3">
-        <v>31</v>
+        <v>629</v>
       </c>
       <c r="D3" t="s">
         <v>80</v>
@@ -5955,18 +5960,18 @@
         <v>107</v>
       </c>
       <c r="I3" s="3">
-        <v>46234.23118008629</v>
+        <v>46244.73807913678</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="18" customHeight="1">
       <c r="A4">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B4">
-        <v>7</v>
+        <v>145</v>
       </c>
       <c r="C4">
-        <v>32</v>
+        <v>630</v>
       </c>
       <c r="D4" t="s">
         <v>81</v>
@@ -5984,18 +5989,18 @@
         <v>107</v>
       </c>
       <c r="I4" s="3">
-        <v>46234.23118008651</v>
+        <v>46244.73807913705</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="18" customHeight="1">
       <c r="A5">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B5">
-        <v>7</v>
+        <v>145</v>
       </c>
       <c r="C5">
-        <v>32</v>
+        <v>630</v>
       </c>
       <c r="D5" t="s">
         <v>82</v>
@@ -6013,18 +6018,18 @@
         <v>107</v>
       </c>
       <c r="I5" s="3">
-        <v>46234.23118008659</v>
+        <v>46244.73807913712</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="18" customHeight="1">
       <c r="A6">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B6">
-        <v>8</v>
+        <v>146</v>
       </c>
       <c r="C6">
-        <v>35</v>
+        <v>633</v>
       </c>
       <c r="D6" t="s">
         <v>79</v>
@@ -6042,18 +6047,18 @@
         <v>107</v>
       </c>
       <c r="I6" s="3">
-        <v>46234.23118008708</v>
+        <v>46244.73807913766</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="18" customHeight="1">
       <c r="A7">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B7">
-        <v>8</v>
+        <v>146</v>
       </c>
       <c r="C7">
-        <v>35</v>
+        <v>633</v>
       </c>
       <c r="D7" t="s">
         <v>83</v>
@@ -6071,18 +6076,18 @@
         <v>107</v>
       </c>
       <c r="I7" s="3">
-        <v>46234.23118008716</v>
+        <v>46244.73807913774</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="18" customHeight="1">
       <c r="A8">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B8">
-        <v>8</v>
+        <v>146</v>
       </c>
       <c r="C8">
-        <v>36</v>
+        <v>634</v>
       </c>
       <c r="D8" t="s">
         <v>81</v>
@@ -6100,18 +6105,18 @@
         <v>107</v>
       </c>
       <c r="I8" s="3">
-        <v>46234.23118008735</v>
+        <v>46244.73807913794</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="18" customHeight="1">
       <c r="A9">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B9">
-        <v>8</v>
+        <v>146</v>
       </c>
       <c r="C9">
-        <v>36</v>
+        <v>634</v>
       </c>
       <c r="D9" t="s">
         <v>82</v>
@@ -6129,18 +6134,18 @@
         <v>107</v>
       </c>
       <c r="I9" s="3">
-        <v>46234.23118008741</v>
+        <v>46244.738079138</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="18" customHeight="1">
       <c r="A10">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B10">
-        <v>9</v>
+        <v>147</v>
       </c>
       <c r="C10">
-        <v>39</v>
+        <v>637</v>
       </c>
       <c r="D10" t="s">
         <v>81</v>
@@ -6158,18 +6163,18 @@
         <v>107</v>
       </c>
       <c r="I10" s="3">
-        <v>46234.23118008792</v>
+        <v>46244.73807913854</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="18" customHeight="1">
       <c r="A11">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B11">
-        <v>7</v>
+        <v>145</v>
       </c>
       <c r="C11">
-        <v>28</v>
+        <v>626</v>
       </c>
       <c r="D11" t="s">
         <v>84</v>
@@ -6187,18 +6192,18 @@
         <v>107</v>
       </c>
       <c r="I11" s="3">
-        <v>46234.2311800957</v>
+        <v>46244.73807914687</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="18" customHeight="1">
       <c r="A12">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B12">
-        <v>7</v>
+        <v>145</v>
       </c>
       <c r="C12">
-        <v>29</v>
+        <v>627</v>
       </c>
       <c r="D12" t="s">
         <v>84</v>
@@ -6216,18 +6221,18 @@
         <v>107</v>
       </c>
       <c r="I12" s="3">
-        <v>46234.2311800959</v>
+        <v>46244.73807914709</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="18" customHeight="1">
       <c r="A13">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B13">
-        <v>9</v>
+        <v>147</v>
       </c>
       <c r="C13">
-        <v>39</v>
+        <v>637</v>
       </c>
       <c r="D13" t="s">
         <v>85</v>
@@ -6245,18 +6250,18 @@
         <v>107</v>
       </c>
       <c r="I13" s="3">
-        <v>46234.23118013208</v>
+        <v>46244.73807918697</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="18" customHeight="1">
       <c r="A14">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="B14">
-        <v>9</v>
+        <v>147</v>
       </c>
       <c r="C14">
-        <v>39</v>
+        <v>637</v>
       </c>
       <c r="D14" t="s">
         <v>85</v>
@@ -6274,12 +6279,12 @@
         <v>107</v>
       </c>
       <c r="I14" s="3">
-        <v>46234.23118013216</v>
+        <v>46244.73807918704</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="18" customHeight="1">
       <c r="A15">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="D15" t="s">
         <v>86</v>
@@ -6297,7 +6302,7 @@
         <v>107</v>
       </c>
       <c r="I15" s="3">
-        <v>46234.23118029253</v>
+        <v>46244.73807935978</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: refresh stable April evidence
</commit_message>
<xml_diff>
--- a/outputs/2026-04/healthcare_ops_kpi_qa_pack_2026_04.xlsx
+++ b/outputs/2026-04/healthcare_ops_kpi_qa_pack_2026_04.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="121">
   <si>
     <t>kpi_name</t>
   </si>
@@ -117,6 +117,9 @@
     <t>variance_pct</t>
   </si>
   <si>
+    <t>kpi_code</t>
+  </si>
+  <si>
     <t>market_name</t>
   </si>
   <si>
@@ -142,6 +145,33 @@
   </si>
   <si>
     <t>Computed for 2026-04 cut `team::TEAM_C`.</t>
+  </si>
+  <si>
+    <t>total_records_received</t>
+  </si>
+  <si>
+    <t>completed_records</t>
+  </si>
+  <si>
+    <t>completion_rate</t>
+  </si>
+  <si>
+    <t>avg_turnaround_days</t>
+  </si>
+  <si>
+    <t>open_backlog_count</t>
+  </si>
+  <si>
+    <t>backlog_over_sla_count</t>
+  </si>
+  <si>
+    <t>qa_issue_rate</t>
+  </si>
+  <si>
+    <t>required_field_completeness_rate</t>
+  </si>
+  <si>
+    <t>unique_npi_rate</t>
   </si>
   <si>
     <t>Chattanooga</t>
@@ -715,12 +745,12 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="18" customHeight="1">
@@ -880,7 +910,7 @@
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1">
@@ -930,13 +960,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P73"/>
+  <dimension ref="A1:Q73"/>
   <sheetFormatPr defaultRowHeight="18" customHeight="1"/>
   <cols>
     <col min="1" max="11" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="18" customHeight="1">
+    <row r="1" spans="1:17" ht="18" customHeight="1">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -977,18 +1007,21 @@
         <v>4</v>
       </c>
       <c r="N1" t="s">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="O1" t="s">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="P1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" ht="18" customHeight="1">
+      <c r="Q1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="18" customHeight="1">
       <c r="A2">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B2">
         <v>20260430</v>
@@ -1015,12 +1048,15 @@
         <v>14</v>
       </c>
       <c r="N2" t="s">
+        <v>42</v>
+      </c>
+      <c r="O2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="18" customHeight="1">
+    <row r="3" spans="1:17" ht="18" customHeight="1">
       <c r="A3">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B3">
         <v>20260430</v>
@@ -1047,12 +1083,15 @@
         <v>14</v>
       </c>
       <c r="N3" t="s">
+        <v>43</v>
+      </c>
+      <c r="O3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="18" customHeight="1">
+    <row r="4" spans="1:17" ht="18" customHeight="1">
       <c r="A4">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B4">
         <v>20260430</v>
@@ -1082,12 +1121,15 @@
         <v>14</v>
       </c>
       <c r="N4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="18" customHeight="1">
+    <row r="5" spans="1:17" ht="18" customHeight="1">
       <c r="A5">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B5">
         <v>20260430</v>
@@ -1114,12 +1156,15 @@
         <v>14</v>
       </c>
       <c r="N5" t="s">
+        <v>45</v>
+      </c>
+      <c r="O5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="18" customHeight="1">
+    <row r="6" spans="1:17" ht="18" customHeight="1">
       <c r="A6">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B6">
         <v>20260430</v>
@@ -1146,12 +1191,15 @@
         <v>14</v>
       </c>
       <c r="N6" t="s">
+        <v>46</v>
+      </c>
+      <c r="O6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="18" customHeight="1">
+    <row r="7" spans="1:17" ht="18" customHeight="1">
       <c r="A7">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B7">
         <v>20260430</v>
@@ -1178,12 +1226,15 @@
         <v>14</v>
       </c>
       <c r="N7" t="s">
+        <v>47</v>
+      </c>
+      <c r="O7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="18" customHeight="1">
+    <row r="8" spans="1:17" ht="18" customHeight="1">
       <c r="A8">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B8">
         <v>20260430</v>
@@ -1213,12 +1264,15 @@
         <v>14</v>
       </c>
       <c r="N8" t="s">
+        <v>48</v>
+      </c>
+      <c r="O8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="18" customHeight="1">
+    <row r="9" spans="1:17" ht="18" customHeight="1">
       <c r="A9">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B9">
         <v>20260430</v>
@@ -1248,12 +1302,15 @@
         <v>14</v>
       </c>
       <c r="N9" t="s">
+        <v>49</v>
+      </c>
+      <c r="O9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="18" customHeight="1">
+    <row r="10" spans="1:17" ht="18" customHeight="1">
       <c r="A10">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B10">
         <v>20260430</v>
@@ -1283,12 +1340,15 @@
         <v>14</v>
       </c>
       <c r="N10" t="s">
+        <v>50</v>
+      </c>
+      <c r="O10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="18" customHeight="1">
+    <row r="11" spans="1:17" ht="18" customHeight="1">
       <c r="A11">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B11">
         <v>20260430</v>
@@ -1315,18 +1375,21 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N11" t="s">
+        <v>42</v>
+      </c>
+      <c r="O11" t="s">
         <v>5</v>
       </c>
-      <c r="O11" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" ht="18" customHeight="1">
+      <c r="P11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" ht="18" customHeight="1">
       <c r="A12">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B12">
         <v>20260430</v>
@@ -1353,18 +1416,21 @@
         <v>0</v>
       </c>
       <c r="M12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N12" t="s">
+        <v>43</v>
+      </c>
+      <c r="O12" t="s">
         <v>6</v>
       </c>
-      <c r="O12" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" ht="18" customHeight="1">
+      <c r="P12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="18" customHeight="1">
       <c r="A13">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B13">
         <v>20260430</v>
@@ -1394,18 +1460,21 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N13" t="s">
+        <v>44</v>
+      </c>
+      <c r="O13" t="s">
         <v>7</v>
       </c>
-      <c r="O13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="18" customHeight="1">
+      <c r="P13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="18" customHeight="1">
       <c r="A14">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B14">
         <v>20260430</v>
@@ -1432,18 +1501,21 @@
         <v>0</v>
       </c>
       <c r="M14" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N14" t="s">
+        <v>45</v>
+      </c>
+      <c r="O14" t="s">
         <v>8</v>
       </c>
-      <c r="O14" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="18" customHeight="1">
+      <c r="P14" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" ht="18" customHeight="1">
       <c r="A15">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B15">
         <v>20260430</v>
@@ -1467,18 +1539,21 @@
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N15" t="s">
+        <v>46</v>
+      </c>
+      <c r="O15" t="s">
         <v>9</v>
       </c>
-      <c r="O15" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="18" customHeight="1">
+      <c r="P15" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="18" customHeight="1">
       <c r="A16">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B16">
         <v>20260430</v>
@@ -1502,18 +1577,21 @@
         <v>0</v>
       </c>
       <c r="M16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N16" t="s">
+        <v>47</v>
+      </c>
+      <c r="O16" t="s">
         <v>10</v>
       </c>
-      <c r="O16" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" ht="18" customHeight="1">
+      <c r="P16" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="18" customHeight="1">
       <c r="A17">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B17">
         <v>20260430</v>
@@ -1540,18 +1618,21 @@
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N17" t="s">
+        <v>48</v>
+      </c>
+      <c r="O17" t="s">
         <v>11</v>
       </c>
-      <c r="O17" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" ht="18" customHeight="1">
+      <c r="P17" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="18" customHeight="1">
       <c r="A18">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B18">
         <v>20260430</v>
@@ -1581,18 +1662,21 @@
         <v>1</v>
       </c>
       <c r="M18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N18" t="s">
+        <v>49</v>
+      </c>
+      <c r="O18" t="s">
         <v>12</v>
       </c>
-      <c r="O18" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" ht="18" customHeight="1">
+      <c r="P18" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" ht="18" customHeight="1">
       <c r="A19">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B19">
         <v>20260430</v>
@@ -1622,18 +1706,21 @@
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N19" t="s">
+        <v>50</v>
+      </c>
+      <c r="O19" t="s">
         <v>13</v>
       </c>
-      <c r="O19" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" ht="18" customHeight="1">
+      <c r="P19" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="18" customHeight="1">
       <c r="A20">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B20">
         <v>20260430</v>
@@ -1660,18 +1747,21 @@
         <v>1</v>
       </c>
       <c r="M20" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N20" t="s">
+        <v>42</v>
+      </c>
+      <c r="O20" t="s">
         <v>5</v>
       </c>
-      <c r="O20" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" ht="18" customHeight="1">
+      <c r="P20" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="18" customHeight="1">
       <c r="A21">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B21">
         <v>20260430</v>
@@ -1695,18 +1785,21 @@
         <v>0</v>
       </c>
       <c r="M21" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N21" t="s">
+        <v>43</v>
+      </c>
+      <c r="O21" t="s">
         <v>6</v>
       </c>
-      <c r="O21" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" ht="18" customHeight="1">
+      <c r="P21" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" ht="18" customHeight="1">
       <c r="A22">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B22">
         <v>20260430</v>
@@ -1733,18 +1826,21 @@
         <v>1</v>
       </c>
       <c r="M22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N22" t="s">
+        <v>44</v>
+      </c>
+      <c r="O22" t="s">
         <v>7</v>
       </c>
-      <c r="O22" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" ht="18" customHeight="1">
+      <c r="P22" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="18" customHeight="1">
       <c r="A23">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B23">
         <v>20260430</v>
@@ -1768,18 +1864,21 @@
         <v>0</v>
       </c>
       <c r="M23" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N23" t="s">
+        <v>45</v>
+      </c>
+      <c r="O23" t="s">
         <v>8</v>
       </c>
-      <c r="O23" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" ht="18" customHeight="1">
+      <c r="P23" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="18" customHeight="1">
       <c r="A24">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B24">
         <v>20260430</v>
@@ -1806,18 +1905,21 @@
         <v>1</v>
       </c>
       <c r="M24" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N24" t="s">
+        <v>46</v>
+      </c>
+      <c r="O24" t="s">
         <v>9</v>
       </c>
-      <c r="O24" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" ht="18" customHeight="1">
+      <c r="P24" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="18" customHeight="1">
       <c r="A25">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B25">
         <v>20260430</v>
@@ -1841,18 +1943,21 @@
         <v>0</v>
       </c>
       <c r="M25" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N25" t="s">
+        <v>47</v>
+      </c>
+      <c r="O25" t="s">
         <v>10</v>
       </c>
-      <c r="O25" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" ht="18" customHeight="1">
+      <c r="P25" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="18" customHeight="1">
       <c r="A26">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B26">
         <v>20260430</v>
@@ -1879,18 +1984,21 @@
         <v>1</v>
       </c>
       <c r="M26" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N26" t="s">
+        <v>48</v>
+      </c>
+      <c r="O26" t="s">
         <v>11</v>
       </c>
-      <c r="O26" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" ht="18" customHeight="1">
+      <c r="P26" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="18" customHeight="1">
       <c r="A27">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B27">
         <v>20260430</v>
@@ -1920,18 +2028,21 @@
         <v>1</v>
       </c>
       <c r="M27" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N27" t="s">
+        <v>49</v>
+      </c>
+      <c r="O27" t="s">
         <v>12</v>
       </c>
-      <c r="O27" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" ht="18" customHeight="1">
+      <c r="P27" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="18" customHeight="1">
       <c r="A28">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B28">
         <v>20260430</v>
@@ -1961,18 +2072,21 @@
         <v>1</v>
       </c>
       <c r="M28" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N28" t="s">
+        <v>50</v>
+      </c>
+      <c r="O28" t="s">
         <v>13</v>
       </c>
-      <c r="O28" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" ht="18" customHeight="1">
+      <c r="P28" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="18" customHeight="1">
       <c r="A29">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B29">
         <v>20260430</v>
@@ -1999,18 +2113,21 @@
         <v>1</v>
       </c>
       <c r="M29" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N29" t="s">
+        <v>42</v>
+      </c>
+      <c r="O29" t="s">
         <v>5</v>
       </c>
-      <c r="O29" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" ht="18" customHeight="1">
+      <c r="P29" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="18" customHeight="1">
       <c r="A30">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B30">
         <v>20260430</v>
@@ -2034,18 +2151,21 @@
         <v>0</v>
       </c>
       <c r="M30" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N30" t="s">
+        <v>43</v>
+      </c>
+      <c r="O30" t="s">
         <v>6</v>
       </c>
-      <c r="O30" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" ht="18" customHeight="1">
+      <c r="P30" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" ht="18" customHeight="1">
       <c r="A31">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B31">
         <v>20260430</v>
@@ -2072,18 +2192,21 @@
         <v>1</v>
       </c>
       <c r="M31" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N31" t="s">
+        <v>44</v>
+      </c>
+      <c r="O31" t="s">
         <v>7</v>
       </c>
-      <c r="O31" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" ht="18" customHeight="1">
+      <c r="P31" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="18" customHeight="1">
       <c r="A32">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B32">
         <v>20260430</v>
@@ -2107,18 +2230,21 @@
         <v>0</v>
       </c>
       <c r="M32" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N32" t="s">
+        <v>45</v>
+      </c>
+      <c r="O32" t="s">
         <v>8</v>
       </c>
-      <c r="O32" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" ht="18" customHeight="1">
+      <c r="P32" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" ht="18" customHeight="1">
       <c r="A33">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B33">
         <v>20260430</v>
@@ -2145,18 +2271,21 @@
         <v>1</v>
       </c>
       <c r="M33" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N33" t="s">
+        <v>46</v>
+      </c>
+      <c r="O33" t="s">
         <v>9</v>
       </c>
-      <c r="O33" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" ht="18" customHeight="1">
+      <c r="P33" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" ht="18" customHeight="1">
       <c r="A34">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B34">
         <v>20260430</v>
@@ -2180,18 +2309,21 @@
         <v>0</v>
       </c>
       <c r="M34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N34" t="s">
+        <v>47</v>
+      </c>
+      <c r="O34" t="s">
         <v>10</v>
       </c>
-      <c r="O34" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16" ht="18" customHeight="1">
+      <c r="P34" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" ht="18" customHeight="1">
       <c r="A35">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B35">
         <v>20260430</v>
@@ -2218,18 +2350,21 @@
         <v>1</v>
       </c>
       <c r="M35" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N35" t="s">
+        <v>48</v>
+      </c>
+      <c r="O35" t="s">
         <v>11</v>
       </c>
-      <c r="O35" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" ht="18" customHeight="1">
+      <c r="P35" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" ht="18" customHeight="1">
       <c r="A36">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B36">
         <v>20260430</v>
@@ -2256,18 +2391,21 @@
         <v>1</v>
       </c>
       <c r="M36" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N36" t="s">
+        <v>49</v>
+      </c>
+      <c r="O36" t="s">
         <v>12</v>
       </c>
-      <c r="O36" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" ht="18" customHeight="1">
+      <c r="P36" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" ht="18" customHeight="1">
       <c r="A37">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B37">
         <v>20260430</v>
@@ -2294,94 +2432,103 @@
         <v>1</v>
       </c>
       <c r="M37" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N37" t="s">
+        <v>50</v>
+      </c>
+      <c r="O37" t="s">
         <v>13</v>
       </c>
-      <c r="O37" t="s">
+      <c r="P37" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" ht="18" customHeight="1">
+      <c r="A38">
+        <v>55</v>
+      </c>
+      <c r="B38">
+        <v>20260430</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="H38">
+        <v>2</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
+        <v>2</v>
+      </c>
+      <c r="M38" t="s">
+        <v>38</v>
+      </c>
+      <c r="N38" t="s">
+        <v>42</v>
+      </c>
+      <c r="O38" t="s">
+        <v>5</v>
+      </c>
+      <c r="P38" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" ht="18" customHeight="1">
+      <c r="A39">
+        <v>55</v>
+      </c>
+      <c r="B39">
+        <v>20260430</v>
+      </c>
+      <c r="C39">
+        <v>2</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="H39">
+        <v>1</v>
+      </c>
+      <c r="I39">
+        <v>0</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
+        <v>1</v>
+      </c>
+      <c r="M39" t="s">
+        <v>38</v>
+      </c>
+      <c r="N39" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="38" spans="1:16" ht="18" customHeight="1">
-      <c r="A38">
-        <v>49</v>
-      </c>
-      <c r="B38">
-        <v>20260430</v>
-      </c>
-      <c r="C38">
-        <v>1</v>
-      </c>
-      <c r="D38">
-        <v>1</v>
-      </c>
-      <c r="F38">
-        <v>2</v>
-      </c>
-      <c r="H38">
-        <v>2</v>
-      </c>
-      <c r="I38">
-        <v>0</v>
-      </c>
-      <c r="J38">
-        <v>0</v>
-      </c>
-      <c r="K38">
-        <v>2</v>
-      </c>
-      <c r="M38" t="s">
-        <v>37</v>
-      </c>
-      <c r="N38" t="s">
-        <v>5</v>
-      </c>
-      <c r="O38" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" ht="18" customHeight="1">
-      <c r="A39">
-        <v>49</v>
-      </c>
-      <c r="B39">
-        <v>20260430</v>
-      </c>
-      <c r="C39">
-        <v>2</v>
-      </c>
-      <c r="D39">
-        <v>1</v>
-      </c>
-      <c r="F39">
-        <v>1</v>
-      </c>
-      <c r="H39">
-        <v>1</v>
-      </c>
-      <c r="I39">
-        <v>0</v>
-      </c>
-      <c r="J39">
-        <v>0</v>
-      </c>
-      <c r="K39">
-        <v>1</v>
-      </c>
-      <c r="M39" t="s">
-        <v>37</v>
-      </c>
-      <c r="N39" t="s">
+      <c r="O39" t="s">
         <v>6</v>
       </c>
-      <c r="O39" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" ht="18" customHeight="1">
+      <c r="P39" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" ht="18" customHeight="1">
       <c r="A40">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B40">
         <v>20260430</v>
@@ -2411,18 +2558,21 @@
         <v>2</v>
       </c>
       <c r="M40" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N40" t="s">
+        <v>44</v>
+      </c>
+      <c r="O40" t="s">
         <v>7</v>
       </c>
-      <c r="O40" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="41" spans="1:16" ht="18" customHeight="1">
+      <c r="P40" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" ht="18" customHeight="1">
       <c r="A41">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B41">
         <v>20260430</v>
@@ -2449,18 +2599,21 @@
         <v>5</v>
       </c>
       <c r="M41" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N41" t="s">
+        <v>45</v>
+      </c>
+      <c r="O41" t="s">
         <v>8</v>
       </c>
-      <c r="O41" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" ht="18" customHeight="1">
+      <c r="P41" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" ht="18" customHeight="1">
       <c r="A42">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B42">
         <v>20260430</v>
@@ -2487,18 +2640,21 @@
         <v>1</v>
       </c>
       <c r="M42" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N42" t="s">
+        <v>46</v>
+      </c>
+      <c r="O42" t="s">
         <v>9</v>
       </c>
-      <c r="O42" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16" ht="18" customHeight="1">
+      <c r="P42" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" ht="18" customHeight="1">
       <c r="A43">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B43">
         <v>20260430</v>
@@ -2525,18 +2681,21 @@
         <v>1</v>
       </c>
       <c r="M43" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N43" t="s">
+        <v>47</v>
+      </c>
+      <c r="O43" t="s">
         <v>10</v>
       </c>
-      <c r="O43" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" ht="18" customHeight="1">
+      <c r="P43" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" ht="18" customHeight="1">
       <c r="A44">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B44">
         <v>20260430</v>
@@ -2566,18 +2725,21 @@
         <v>2</v>
       </c>
       <c r="M44" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N44" t="s">
+        <v>48</v>
+      </c>
+      <c r="O44" t="s">
         <v>11</v>
       </c>
-      <c r="O44" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="45" spans="1:16" ht="18" customHeight="1">
+      <c r="P44" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" ht="18" customHeight="1">
       <c r="A45">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B45">
         <v>20260430</v>
@@ -2607,18 +2769,21 @@
         <v>2</v>
       </c>
       <c r="M45" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N45" t="s">
+        <v>49</v>
+      </c>
+      <c r="O45" t="s">
         <v>12</v>
       </c>
-      <c r="O45" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" ht="18" customHeight="1">
+      <c r="P45" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" ht="18" customHeight="1">
       <c r="A46">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B46">
         <v>20260430</v>
@@ -2648,18 +2813,21 @@
         <v>2</v>
       </c>
       <c r="M46" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N46" t="s">
+        <v>50</v>
+      </c>
+      <c r="O46" t="s">
         <v>13</v>
       </c>
-      <c r="O46" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" ht="18" customHeight="1">
+      <c r="P46" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" ht="18" customHeight="1">
       <c r="A47">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B47">
         <v>20260430</v>
@@ -2686,18 +2854,21 @@
         <v>2</v>
       </c>
       <c r="M47" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N47" t="s">
+        <v>42</v>
+      </c>
+      <c r="O47" t="s">
         <v>5</v>
       </c>
-      <c r="P47" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" ht="18" customHeight="1">
+      <c r="Q47" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17" ht="18" customHeight="1">
       <c r="A48">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B48">
         <v>20260430</v>
@@ -2724,18 +2895,21 @@
         <v>1</v>
       </c>
       <c r="M48" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N48" t="s">
+        <v>43</v>
+      </c>
+      <c r="O48" t="s">
         <v>6</v>
       </c>
-      <c r="P48" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="49" spans="1:16" ht="18" customHeight="1">
+      <c r="Q48" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" ht="18" customHeight="1">
       <c r="A49">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B49">
         <v>20260430</v>
@@ -2765,18 +2939,21 @@
         <v>2</v>
       </c>
       <c r="M49" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N49" t="s">
+        <v>44</v>
+      </c>
+      <c r="O49" t="s">
         <v>7</v>
       </c>
-      <c r="P49" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="50" spans="1:16" ht="18" customHeight="1">
+      <c r="Q49" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" ht="18" customHeight="1">
       <c r="A50">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B50">
         <v>20260430</v>
@@ -2803,18 +2980,21 @@
         <v>5</v>
       </c>
       <c r="M50" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N50" t="s">
+        <v>45</v>
+      </c>
+      <c r="O50" t="s">
         <v>8</v>
       </c>
-      <c r="P50" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="51" spans="1:16" ht="18" customHeight="1">
+      <c r="Q50" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" ht="18" customHeight="1">
       <c r="A51">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B51">
         <v>20260430</v>
@@ -2841,18 +3021,21 @@
         <v>1</v>
       </c>
       <c r="M51" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N51" t="s">
+        <v>46</v>
+      </c>
+      <c r="O51" t="s">
         <v>9</v>
       </c>
-      <c r="P51" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="52" spans="1:16" ht="18" customHeight="1">
+      <c r="Q51" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" ht="18" customHeight="1">
       <c r="A52">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B52">
         <v>20260430</v>
@@ -2879,18 +3062,21 @@
         <v>1</v>
       </c>
       <c r="M52" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N52" t="s">
+        <v>47</v>
+      </c>
+      <c r="O52" t="s">
         <v>10</v>
       </c>
-      <c r="P52" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="53" spans="1:16" ht="18" customHeight="1">
+      <c r="Q52" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17" ht="18" customHeight="1">
       <c r="A53">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B53">
         <v>20260430</v>
@@ -2920,18 +3106,21 @@
         <v>2</v>
       </c>
       <c r="M53" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N53" t="s">
+        <v>48</v>
+      </c>
+      <c r="O53" t="s">
         <v>11</v>
       </c>
-      <c r="P53" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="54" spans="1:16" ht="18" customHeight="1">
+      <c r="Q53" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" ht="18" customHeight="1">
       <c r="A54">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B54">
         <v>20260430</v>
@@ -2961,18 +3150,21 @@
         <v>2</v>
       </c>
       <c r="M54" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N54" t="s">
+        <v>49</v>
+      </c>
+      <c r="O54" t="s">
         <v>12</v>
       </c>
-      <c r="P54" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="55" spans="1:16" ht="18" customHeight="1">
+      <c r="Q54" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17" ht="18" customHeight="1">
       <c r="A55">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B55">
         <v>20260430</v>
@@ -3002,18 +3194,21 @@
         <v>2</v>
       </c>
       <c r="M55" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N55" t="s">
+        <v>50</v>
+      </c>
+      <c r="O55" t="s">
         <v>13</v>
       </c>
-      <c r="P55" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="56" spans="1:16" ht="18" customHeight="1">
+      <c r="Q55" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" ht="18" customHeight="1">
       <c r="A56">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B56">
         <v>20260430</v>
@@ -3040,18 +3235,21 @@
         <v>2</v>
       </c>
       <c r="M56" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N56" t="s">
+        <v>42</v>
+      </c>
+      <c r="O56" t="s">
         <v>5</v>
       </c>
-      <c r="P56" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="57" spans="1:16" ht="18" customHeight="1">
+      <c r="Q56" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17" ht="18" customHeight="1">
       <c r="A57">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B57">
         <v>20260430</v>
@@ -3075,18 +3273,21 @@
         <v>0</v>
       </c>
       <c r="M57" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N57" t="s">
+        <v>43</v>
+      </c>
+      <c r="O57" t="s">
         <v>6</v>
       </c>
-      <c r="P57" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="58" spans="1:16" ht="18" customHeight="1">
+      <c r="Q57" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17" ht="18" customHeight="1">
       <c r="A58">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B58">
         <v>20260430</v>
@@ -3113,18 +3314,21 @@
         <v>2</v>
       </c>
       <c r="M58" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N58" t="s">
+        <v>44</v>
+      </c>
+      <c r="O58" t="s">
         <v>7</v>
       </c>
-      <c r="P58" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="59" spans="1:16" ht="18" customHeight="1">
+      <c r="Q58" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17" ht="18" customHeight="1">
       <c r="A59">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B59">
         <v>20260430</v>
@@ -3148,18 +3352,21 @@
         <v>0</v>
       </c>
       <c r="M59" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N59" t="s">
+        <v>45</v>
+      </c>
+      <c r="O59" t="s">
         <v>8</v>
       </c>
-      <c r="P59" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="60" spans="1:16" ht="18" customHeight="1">
+      <c r="Q59" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17" ht="18" customHeight="1">
       <c r="A60">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B60">
         <v>20260430</v>
@@ -3186,18 +3393,21 @@
         <v>2</v>
       </c>
       <c r="M60" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N60" t="s">
+        <v>46</v>
+      </c>
+      <c r="O60" t="s">
         <v>9</v>
       </c>
-      <c r="P60" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="61" spans="1:16" ht="18" customHeight="1">
+      <c r="Q60" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17" ht="18" customHeight="1">
       <c r="A61">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B61">
         <v>20260430</v>
@@ -3221,18 +3431,21 @@
         <v>0</v>
       </c>
       <c r="M61" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N61" t="s">
+        <v>47</v>
+      </c>
+      <c r="O61" t="s">
         <v>10</v>
       </c>
-      <c r="P61" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="62" spans="1:16" ht="18" customHeight="1">
+      <c r="Q61" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17" ht="18" customHeight="1">
       <c r="A62">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B62">
         <v>20260430</v>
@@ -3259,18 +3472,21 @@
         <v>2</v>
       </c>
       <c r="M62" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N62" t="s">
+        <v>48</v>
+      </c>
+      <c r="O62" t="s">
         <v>11</v>
       </c>
-      <c r="P62" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="63" spans="1:16" ht="18" customHeight="1">
+      <c r="Q62" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17" ht="18" customHeight="1">
       <c r="A63">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B63">
         <v>20260430</v>
@@ -3300,18 +3516,21 @@
         <v>2</v>
       </c>
       <c r="M63" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N63" t="s">
+        <v>49</v>
+      </c>
+      <c r="O63" t="s">
         <v>12</v>
       </c>
-      <c r="P63" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="64" spans="1:16" ht="18" customHeight="1">
+      <c r="Q63" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="64" spans="1:17" ht="18" customHeight="1">
       <c r="A64">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B64">
         <v>20260430</v>
@@ -3341,18 +3560,21 @@
         <v>2</v>
       </c>
       <c r="M64" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N64" t="s">
+        <v>50</v>
+      </c>
+      <c r="O64" t="s">
         <v>13</v>
       </c>
-      <c r="P64" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="65" spans="1:16" ht="18" customHeight="1">
+      <c r="Q64" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="65" spans="1:17" ht="18" customHeight="1">
       <c r="A65">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B65">
         <v>20260430</v>
@@ -3379,18 +3601,21 @@
         <v>1</v>
       </c>
       <c r="M65" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N65" t="s">
+        <v>42</v>
+      </c>
+      <c r="O65" t="s">
         <v>5</v>
       </c>
-      <c r="P65" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="66" spans="1:16" ht="18" customHeight="1">
+      <c r="Q65" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="66" spans="1:17" ht="18" customHeight="1">
       <c r="A66">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B66">
         <v>20260430</v>
@@ -3417,18 +3642,21 @@
         <v>0</v>
       </c>
       <c r="M66" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N66" t="s">
+        <v>43</v>
+      </c>
+      <c r="O66" t="s">
         <v>6</v>
       </c>
-      <c r="P66" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="67" spans="1:16" ht="18" customHeight="1">
+      <c r="Q66" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="67" spans="1:17" ht="18" customHeight="1">
       <c r="A67">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B67">
         <v>20260430</v>
@@ -3458,18 +3686,21 @@
         <v>1</v>
       </c>
       <c r="M67" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N67" t="s">
+        <v>44</v>
+      </c>
+      <c r="O67" t="s">
         <v>7</v>
       </c>
-      <c r="P67" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="68" spans="1:16" ht="18" customHeight="1">
+      <c r="Q67" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="68" spans="1:17" ht="18" customHeight="1">
       <c r="A68">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B68">
         <v>20260430</v>
@@ -3496,18 +3727,21 @@
         <v>0</v>
       </c>
       <c r="M68" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N68" t="s">
+        <v>45</v>
+      </c>
+      <c r="O68" t="s">
         <v>8</v>
       </c>
-      <c r="P68" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="69" spans="1:16" ht="18" customHeight="1">
+      <c r="Q68" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="69" spans="1:17" ht="18" customHeight="1">
       <c r="A69">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B69">
         <v>20260430</v>
@@ -3531,18 +3765,21 @@
         <v>1</v>
       </c>
       <c r="M69" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N69" t="s">
+        <v>46</v>
+      </c>
+      <c r="O69" t="s">
         <v>9</v>
       </c>
-      <c r="P69" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="70" spans="1:16" ht="18" customHeight="1">
+      <c r="Q69" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="70" spans="1:17" ht="18" customHeight="1">
       <c r="A70">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B70">
         <v>20260430</v>
@@ -3566,18 +3803,21 @@
         <v>0</v>
       </c>
       <c r="M70" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N70" t="s">
+        <v>47</v>
+      </c>
+      <c r="O70" t="s">
         <v>10</v>
       </c>
-      <c r="P70" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="71" spans="1:16" ht="18" customHeight="1">
+      <c r="Q70" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="71" spans="1:17" ht="18" customHeight="1">
       <c r="A71">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B71">
         <v>20260430</v>
@@ -3604,18 +3844,21 @@
         <v>1</v>
       </c>
       <c r="M71" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N71" t="s">
+        <v>48</v>
+      </c>
+      <c r="O71" t="s">
         <v>11</v>
       </c>
-      <c r="P71" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="72" spans="1:16" ht="18" customHeight="1">
+      <c r="Q71" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="72" spans="1:17" ht="18" customHeight="1">
       <c r="A72">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B72">
         <v>20260430</v>
@@ -3645,18 +3888,21 @@
         <v>1</v>
       </c>
       <c r="M72" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N72" t="s">
+        <v>49</v>
+      </c>
+      <c r="O72" t="s">
         <v>12</v>
       </c>
-      <c r="P72" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="73" spans="1:16" ht="18" customHeight="1">
+      <c r="Q72" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="73" spans="1:17" ht="18" customHeight="1">
       <c r="A73">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B73">
         <v>20260430</v>
@@ -3686,13 +3932,16 @@
         <v>1</v>
       </c>
       <c r="M73" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N73" t="s">
+        <v>50</v>
+      </c>
+      <c r="O73" t="s">
         <v>13</v>
       </c>
-      <c r="P73" t="s">
-        <v>47</v>
+      <c r="Q73" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -3710,10 +3959,10 @@
   <sheetData>
     <row r="1" spans="1:8" ht="18" customHeight="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -3889,7 +4138,7 @@
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1">
       <c r="A11" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C11" t="s">
         <v>5</v>
@@ -3909,7 +4158,7 @@
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1">
       <c r="A12" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C12" t="s">
         <v>6</v>
@@ -3929,7 +4178,7 @@
     </row>
     <row r="13" spans="1:8" ht="18" customHeight="1">
       <c r="A13" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C13" t="s">
         <v>7</v>
@@ -3949,7 +4198,7 @@
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1">
       <c r="A14" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C14" t="s">
         <v>8</v>
@@ -3969,7 +4218,7 @@
     </row>
     <row r="15" spans="1:8" ht="18" customHeight="1">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C15" t="s">
         <v>9</v>
@@ -3986,7 +4235,7 @@
     </row>
     <row r="16" spans="1:8" ht="18" customHeight="1">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C16" t="s">
         <v>10</v>
@@ -4003,7 +4252,7 @@
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C17" t="s">
         <v>11</v>
@@ -4020,7 +4269,7 @@
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1">
       <c r="A18" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C18" t="s">
         <v>12</v>
@@ -4040,7 +4289,7 @@
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1">
       <c r="A19" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C19" t="s">
         <v>13</v>
@@ -4060,7 +4309,7 @@
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1">
       <c r="A20" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="C20" t="s">
         <v>5</v>
@@ -4080,7 +4329,7 @@
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1">
       <c r="A21" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="C21" t="s">
         <v>6</v>
@@ -4097,7 +4346,7 @@
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1">
       <c r="A22" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="C22" t="s">
         <v>7</v>
@@ -4114,7 +4363,7 @@
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1">
       <c r="A23" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="C23" t="s">
         <v>8</v>
@@ -4131,7 +4380,7 @@
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1">
       <c r="A24" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="C24" t="s">
         <v>9</v>
@@ -4151,7 +4400,7 @@
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1">
       <c r="A25" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="C25" t="s">
         <v>10</v>
@@ -4168,7 +4417,7 @@
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1">
       <c r="A26" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="C26" t="s">
         <v>11</v>
@@ -4185,7 +4434,7 @@
     </row>
     <row r="27" spans="1:8" ht="18" customHeight="1">
       <c r="A27" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="C27" t="s">
         <v>12</v>
@@ -4205,7 +4454,7 @@
     </row>
     <row r="28" spans="1:8" ht="18" customHeight="1">
       <c r="A28" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="C28" t="s">
         <v>13</v>
@@ -4225,7 +4474,7 @@
     </row>
     <row r="29" spans="1:8" ht="18" customHeight="1">
       <c r="A29" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C29" t="s">
         <v>5</v>
@@ -4245,7 +4494,7 @@
     </row>
     <row r="30" spans="1:8" ht="18" customHeight="1">
       <c r="A30" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C30" t="s">
         <v>6</v>
@@ -4262,7 +4511,7 @@
     </row>
     <row r="31" spans="1:8" ht="18" customHeight="1">
       <c r="A31" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C31" t="s">
         <v>7</v>
@@ -4279,7 +4528,7 @@
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1">
       <c r="A32" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C32" t="s">
         <v>8</v>
@@ -4296,7 +4545,7 @@
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1">
       <c r="A33" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C33" t="s">
         <v>9</v>
@@ -4316,7 +4565,7 @@
     </row>
     <row r="34" spans="1:8" ht="18" customHeight="1">
       <c r="A34" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C34" t="s">
         <v>10</v>
@@ -4333,7 +4582,7 @@
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1">
       <c r="A35" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C35" t="s">
         <v>11</v>
@@ -4350,7 +4599,7 @@
     </row>
     <row r="36" spans="1:8" ht="18" customHeight="1">
       <c r="A36" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C36" t="s">
         <v>12</v>
@@ -4367,7 +4616,7 @@
     </row>
     <row r="37" spans="1:8" ht="18" customHeight="1">
       <c r="A37" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C37" t="s">
         <v>13</v>
@@ -4384,7 +4633,7 @@
     </row>
     <row r="38" spans="1:8" ht="18" customHeight="1">
       <c r="A38" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C38" t="s">
         <v>5</v>
@@ -4404,7 +4653,7 @@
     </row>
     <row r="39" spans="1:8" ht="18" customHeight="1">
       <c r="A39" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C39" t="s">
         <v>6</v>
@@ -4424,7 +4673,7 @@
     </row>
     <row r="40" spans="1:8" ht="18" customHeight="1">
       <c r="A40" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C40" t="s">
         <v>7</v>
@@ -4444,7 +4693,7 @@
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1">
       <c r="A41" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C41" t="s">
         <v>8</v>
@@ -4464,7 +4713,7 @@
     </row>
     <row r="42" spans="1:8" ht="18" customHeight="1">
       <c r="A42" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C42" t="s">
         <v>9</v>
@@ -4484,7 +4733,7 @@
     </row>
     <row r="43" spans="1:8" ht="18" customHeight="1">
       <c r="A43" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C43" t="s">
         <v>10</v>
@@ -4504,7 +4753,7 @@
     </row>
     <row r="44" spans="1:8" ht="18" customHeight="1">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C44" t="s">
         <v>11</v>
@@ -4524,7 +4773,7 @@
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1">
       <c r="A45" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C45" t="s">
         <v>12</v>
@@ -4544,7 +4793,7 @@
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1">
       <c r="A46" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C46" t="s">
         <v>13</v>
@@ -4564,7 +4813,7 @@
     </row>
     <row r="47" spans="1:8" ht="18" customHeight="1">
       <c r="B47" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C47" t="s">
         <v>5</v>
@@ -4584,7 +4833,7 @@
     </row>
     <row r="48" spans="1:8" ht="18" customHeight="1">
       <c r="B48" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C48" t="s">
         <v>6</v>
@@ -4604,7 +4853,7 @@
     </row>
     <row r="49" spans="2:8" ht="18" customHeight="1">
       <c r="B49" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C49" t="s">
         <v>7</v>
@@ -4624,7 +4873,7 @@
     </row>
     <row r="50" spans="2:8" ht="18" customHeight="1">
       <c r="B50" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C50" t="s">
         <v>8</v>
@@ -4644,7 +4893,7 @@
     </row>
     <row r="51" spans="2:8" ht="18" customHeight="1">
       <c r="B51" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C51" t="s">
         <v>9</v>
@@ -4664,7 +4913,7 @@
     </row>
     <row r="52" spans="2:8" ht="18" customHeight="1">
       <c r="B52" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C52" t="s">
         <v>10</v>
@@ -4684,7 +4933,7 @@
     </row>
     <row r="53" spans="2:8" ht="18" customHeight="1">
       <c r="B53" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C53" t="s">
         <v>11</v>
@@ -4704,7 +4953,7 @@
     </row>
     <row r="54" spans="2:8" ht="18" customHeight="1">
       <c r="B54" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C54" t="s">
         <v>12</v>
@@ -4724,7 +4973,7 @@
     </row>
     <row r="55" spans="2:8" ht="18" customHeight="1">
       <c r="B55" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C55" t="s">
         <v>13</v>
@@ -4744,7 +4993,7 @@
     </row>
     <row r="56" spans="2:8" ht="18" customHeight="1">
       <c r="B56" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C56" t="s">
         <v>5</v>
@@ -4764,7 +5013,7 @@
     </row>
     <row r="57" spans="2:8" ht="18" customHeight="1">
       <c r="B57" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C57" t="s">
         <v>6</v>
@@ -4781,7 +5030,7 @@
     </row>
     <row r="58" spans="2:8" ht="18" customHeight="1">
       <c r="B58" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C58" t="s">
         <v>7</v>
@@ -4798,7 +5047,7 @@
     </row>
     <row r="59" spans="2:8" ht="18" customHeight="1">
       <c r="B59" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C59" t="s">
         <v>8</v>
@@ -4815,7 +5064,7 @@
     </row>
     <row r="60" spans="2:8" ht="18" customHeight="1">
       <c r="B60" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C60" t="s">
         <v>9</v>
@@ -4835,7 +5084,7 @@
     </row>
     <row r="61" spans="2:8" ht="18" customHeight="1">
       <c r="B61" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C61" t="s">
         <v>10</v>
@@ -4852,7 +5101,7 @@
     </row>
     <row r="62" spans="2:8" ht="18" customHeight="1">
       <c r="B62" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C62" t="s">
         <v>11</v>
@@ -4869,7 +5118,7 @@
     </row>
     <row r="63" spans="2:8" ht="18" customHeight="1">
       <c r="B63" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C63" t="s">
         <v>12</v>
@@ -4889,7 +5138,7 @@
     </row>
     <row r="64" spans="2:8" ht="18" customHeight="1">
       <c r="B64" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C64" t="s">
         <v>13</v>
@@ -4909,7 +5158,7 @@
     </row>
     <row r="65" spans="2:8" ht="18" customHeight="1">
       <c r="B65" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C65" t="s">
         <v>5</v>
@@ -4929,7 +5178,7 @@
     </row>
     <row r="66" spans="2:8" ht="18" customHeight="1">
       <c r="B66" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C66" t="s">
         <v>6</v>
@@ -4949,7 +5198,7 @@
     </row>
     <row r="67" spans="2:8" ht="18" customHeight="1">
       <c r="B67" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C67" t="s">
         <v>7</v>
@@ -4969,7 +5218,7 @@
     </row>
     <row r="68" spans="2:8" ht="18" customHeight="1">
       <c r="B68" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C68" t="s">
         <v>8</v>
@@ -4989,7 +5238,7 @@
     </row>
     <row r="69" spans="2:8" ht="18" customHeight="1">
       <c r="B69" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C69" t="s">
         <v>9</v>
@@ -5006,7 +5255,7 @@
     </row>
     <row r="70" spans="2:8" ht="18" customHeight="1">
       <c r="B70" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C70" t="s">
         <v>10</v>
@@ -5023,7 +5272,7 @@
     </row>
     <row r="71" spans="2:8" ht="18" customHeight="1">
       <c r="B71" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C71" t="s">
         <v>11</v>
@@ -5040,7 +5289,7 @@
     </row>
     <row r="72" spans="2:8" ht="18" customHeight="1">
       <c r="B72" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C72" t="s">
         <v>12</v>
@@ -5060,7 +5309,7 @@
     </row>
     <row r="73" spans="2:8" ht="18" customHeight="1">
       <c r="B73" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C73" t="s">
         <v>13</v>
@@ -5096,22 +5345,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D1" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="E1" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="F1" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="G1" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1">
@@ -5128,7 +5377,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1">
@@ -5136,7 +5385,7 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -5148,7 +5397,7 @@
         <v>2</v>
       </c>
       <c r="G3" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="18" customHeight="1">
@@ -5156,7 +5405,7 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="D4">
         <v>2</v>
@@ -5168,7 +5417,7 @@
         <v>2</v>
       </c>
       <c r="G4" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="18" customHeight="1">
@@ -5176,7 +5425,7 @@
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -5188,7 +5437,7 @@
         <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="18" customHeight="1">
@@ -5196,7 +5445,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="D6">
         <v>2</v>
@@ -5208,7 +5457,7 @@
         <v>2</v>
       </c>
       <c r="G6" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="18" customHeight="1">
@@ -5216,7 +5465,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -5228,7 +5477,7 @@
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="18" customHeight="1">
@@ -5236,7 +5485,7 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -5248,7 +5497,7 @@
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="18" customHeight="1">
@@ -5256,7 +5505,7 @@
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -5268,7 +5517,7 @@
         <v>1</v>
       </c>
       <c r="G9" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="18" customHeight="1">
@@ -5285,7 +5534,7 @@
         <v>2</v>
       </c>
       <c r="G10" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="18" customHeight="1">
@@ -5293,7 +5542,7 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="D11">
         <v>0.6666666666666666</v>
@@ -5305,7 +5554,7 @@
         <v>1</v>
       </c>
       <c r="G11" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="18" customHeight="1">
@@ -5313,7 +5562,7 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -5325,7 +5574,7 @@
         <v>0</v>
       </c>
       <c r="G12" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="18" customHeight="1">
@@ -5333,7 +5582,7 @@
         <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="D13">
         <v>0.3333333333333333</v>
@@ -5345,7 +5594,7 @@
         <v>1</v>
       </c>
       <c r="G13" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="18" customHeight="1">
@@ -5353,7 +5602,7 @@
         <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="D14">
         <v>0.6666666666666666</v>
@@ -5365,7 +5614,7 @@
         <v>1</v>
       </c>
       <c r="G14" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="18" customHeight="1">
@@ -5373,7 +5622,7 @@
         <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -5385,7 +5634,7 @@
         <v>0</v>
       </c>
       <c r="G15" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="18" customHeight="1">
@@ -5393,7 +5642,7 @@
         <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="D16">
         <v>0</v>
@@ -5405,7 +5654,7 @@
         <v>0</v>
       </c>
       <c r="G16" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="18" customHeight="1">
@@ -5413,7 +5662,7 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="D17">
         <v>0.3333333333333333</v>
@@ -5425,7 +5674,7 @@
         <v>1</v>
       </c>
       <c r="G17" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="18" customHeight="1">
@@ -5442,7 +5691,7 @@
         <v>5</v>
       </c>
       <c r="G18" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1">
@@ -5450,7 +5699,7 @@
         <v>9</v>
       </c>
       <c r="C19" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="D19">
         <v>1.333333333333333</v>
@@ -5462,7 +5711,7 @@
         <v>2</v>
       </c>
       <c r="G19" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="18" customHeight="1">
@@ -5470,7 +5719,7 @@
         <v>9</v>
       </c>
       <c r="C20" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="D20">
         <v>2</v>
@@ -5482,7 +5731,7 @@
         <v>2</v>
       </c>
       <c r="G20" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="18" customHeight="1">
@@ -5490,7 +5739,7 @@
         <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="D21">
         <v>0.6666666666666666</v>
@@ -5502,7 +5751,7 @@
         <v>1</v>
       </c>
       <c r="G21" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="18" customHeight="1">
@@ -5510,7 +5759,7 @@
         <v>9</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="D22">
         <v>1.333333333333333</v>
@@ -5522,7 +5771,7 @@
         <v>2</v>
       </c>
       <c r="G22" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="18" customHeight="1">
@@ -5530,7 +5779,7 @@
         <v>9</v>
       </c>
       <c r="B23" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -5542,7 +5791,7 @@
         <v>1</v>
       </c>
       <c r="G23" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="18" customHeight="1">
@@ -5550,7 +5799,7 @@
         <v>9</v>
       </c>
       <c r="B24" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -5562,7 +5811,7 @@
         <v>1</v>
       </c>
       <c r="G24" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="18" customHeight="1">
@@ -5570,7 +5819,7 @@
         <v>9</v>
       </c>
       <c r="B25" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="D25">
         <v>0.6666666666666666</v>
@@ -5582,7 +5831,7 @@
         <v>1</v>
       </c>
       <c r="G25" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="18" customHeight="1">
@@ -5599,7 +5848,7 @@
         <v>1</v>
       </c>
       <c r="G26" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="18" customHeight="1">
@@ -5607,7 +5856,7 @@
         <v>10</v>
       </c>
       <c r="C27" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -5619,7 +5868,7 @@
         <v>1</v>
       </c>
       <c r="G27" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="18" customHeight="1">
@@ -5627,7 +5876,7 @@
         <v>10</v>
       </c>
       <c r="C28" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="D28">
         <v>0</v>
@@ -5639,7 +5888,7 @@
         <v>0</v>
       </c>
       <c r="G28" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1">
@@ -5647,7 +5896,7 @@
         <v>10</v>
       </c>
       <c r="C29" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="D29">
         <v>0</v>
@@ -5659,7 +5908,7 @@
         <v>0</v>
       </c>
       <c r="G29" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="18" customHeight="1">
@@ -5667,7 +5916,7 @@
         <v>10</v>
       </c>
       <c r="B30" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="D30">
         <v>1</v>
@@ -5679,7 +5928,7 @@
         <v>1</v>
       </c>
       <c r="G30" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="18" customHeight="1">
@@ -5687,7 +5936,7 @@
         <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -5699,7 +5948,7 @@
         <v>0</v>
       </c>
       <c r="G31" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1">
@@ -5707,7 +5956,7 @@
         <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -5719,7 +5968,7 @@
         <v>0</v>
       </c>
       <c r="G32" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="18" customHeight="1">
@@ -5727,7 +5976,7 @@
         <v>10</v>
       </c>
       <c r="B33" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="D33">
         <v>0</v>
@@ -5739,7 +5988,7 @@
         <v>0</v>
       </c>
       <c r="G33" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -5757,10 +6006,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" customHeight="1">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="B1" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="18" customHeight="1">
@@ -5768,20 +6017,20 @@
         <v>23</v>
       </c>
       <c r="B2">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18" customHeight="1">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="18" customHeight="1">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="B4">
         <v>13</v>
@@ -5789,7 +6038,7 @@
     </row>
     <row r="5" spans="1:3" ht="18" customHeight="1">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="B5">
         <v>5</v>
@@ -5797,7 +6046,7 @@
     </row>
     <row r="6" spans="1:3" ht="18" customHeight="1">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B6">
         <v>14</v>
@@ -5805,7 +6054,7 @@
     </row>
     <row r="7" spans="1:3" ht="18" customHeight="1">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="B7">
         <v>72</v>
@@ -5813,7 +6062,7 @@
     </row>
     <row r="8" spans="1:3" ht="18" customHeight="1">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B8">
         <v>32</v>
@@ -5821,21 +6070,21 @@
     </row>
     <row r="11" spans="1:3" ht="18" customHeight="1">
       <c r="A11" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="B11" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="18" customHeight="1">
       <c r="A12" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C12">
         <v>6</v>
@@ -5843,10 +6092,10 @@
     </row>
     <row r="13" spans="1:3" ht="18" customHeight="1">
       <c r="A13" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="B13" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="C13">
         <v>4</v>
@@ -5854,10 +6103,10 @@
     </row>
     <row r="14" spans="1:3" ht="18" customHeight="1">
       <c r="A14" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="C14">
         <v>3</v>
@@ -5881,428 +6130,428 @@
         <v>23</v>
       </c>
       <c r="B1" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C1" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="D1" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="E1" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="F1" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="G1" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="H1" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="I1" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="18" customHeight="1">
       <c r="A2">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B2">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="C2">
-        <v>628</v>
+        <v>706</v>
       </c>
       <c r="D2" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="E2" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="F2" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="G2" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="H2" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I2" s="3">
-        <v>46244.73807913656</v>
+        <v>46245.2551947109</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="18" customHeight="1">
       <c r="A3">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B3">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="C3">
-        <v>629</v>
+        <v>707</v>
       </c>
       <c r="D3" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="E3" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="F3" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G3" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="H3" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I3" s="3">
-        <v>46244.73807913678</v>
+        <v>46245.2551947111</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="18" customHeight="1">
       <c r="A4">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B4">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="C4">
-        <v>630</v>
+        <v>708</v>
       </c>
       <c r="D4" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="E4" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F4" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="G4" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="H4" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I4" s="3">
-        <v>46244.73807913705</v>
+        <v>46245.25519471135</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="18" customHeight="1">
       <c r="A5">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B5">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="C5">
-        <v>630</v>
+        <v>708</v>
       </c>
       <c r="D5" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="E5" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F5" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="G5" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H5" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I5" s="3">
-        <v>46244.73807913712</v>
+        <v>46245.2551947114</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="18" customHeight="1">
       <c r="A6">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B6">
-        <v>146</v>
+        <v>164</v>
       </c>
       <c r="C6">
-        <v>633</v>
+        <v>711</v>
       </c>
       <c r="D6" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="E6" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="F6" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="G6" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="H6" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I6" s="3">
-        <v>46244.73807913766</v>
+        <v>46245.2551947119</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="18" customHeight="1">
       <c r="A7">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B7">
-        <v>146</v>
+        <v>164</v>
       </c>
       <c r="C7">
-        <v>633</v>
+        <v>711</v>
       </c>
       <c r="D7" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="E7" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="F7" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="G7" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="H7" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I7" s="3">
-        <v>46244.73807913774</v>
+        <v>46245.25519471198</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="18" customHeight="1">
       <c r="A8">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B8">
-        <v>146</v>
+        <v>164</v>
       </c>
       <c r="C8">
-        <v>634</v>
+        <v>712</v>
       </c>
       <c r="D8" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="E8" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F8" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="G8" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="H8" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I8" s="3">
-        <v>46244.73807913794</v>
+        <v>46245.25519471216</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="18" customHeight="1">
       <c r="A9">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B9">
-        <v>146</v>
+        <v>164</v>
       </c>
       <c r="C9">
-        <v>634</v>
+        <v>712</v>
       </c>
       <c r="D9" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="E9" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F9" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="G9" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H9" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I9" s="3">
-        <v>46244.738079138</v>
+        <v>46245.25519471222</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="18" customHeight="1">
       <c r="A10">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B10">
-        <v>147</v>
+        <v>165</v>
       </c>
       <c r="C10">
-        <v>637</v>
+        <v>715</v>
       </c>
       <c r="D10" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="E10" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F10" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="G10" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="H10" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I10" s="3">
-        <v>46244.73807913854</v>
+        <v>46245.25519471271</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="18" customHeight="1">
       <c r="A11">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B11">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="C11">
-        <v>626</v>
+        <v>704</v>
       </c>
       <c r="D11" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="E11" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F11" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="G11" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="H11" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I11" s="3">
-        <v>46244.73807914687</v>
+        <v>46245.25519472045</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="18" customHeight="1">
       <c r="A12">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B12">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="C12">
-        <v>627</v>
+        <v>705</v>
       </c>
       <c r="D12" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="E12" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F12" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="G12" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="H12" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I12" s="3">
-        <v>46244.73807914709</v>
+        <v>46245.25519472066</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="18" customHeight="1">
       <c r="A13">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B13">
-        <v>147</v>
+        <v>165</v>
       </c>
       <c r="C13">
-        <v>637</v>
+        <v>715</v>
       </c>
       <c r="D13" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="E13" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F13" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="G13" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="H13" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I13" s="3">
-        <v>46244.73807918697</v>
+        <v>46245.25519475734</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="18" customHeight="1">
       <c r="A14">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B14">
-        <v>147</v>
+        <v>165</v>
       </c>
       <c r="C14">
-        <v>637</v>
+        <v>715</v>
       </c>
       <c r="D14" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="E14" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F14" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="G14" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="H14" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I14" s="3">
-        <v>46244.73807918704</v>
+        <v>46245.25519475741</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="18" customHeight="1">
       <c r="A15">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D15" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="E15" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F15" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="G15" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="H15" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="I15" s="3">
-        <v>46244.73807935978</v>
+        <v>46245.25519491682</v>
       </c>
     </row>
   </sheetData>

</xml_diff>